<commit_message>
Experiment 2 rerun (Conformist bias)
</commit_message>
<xml_diff>
--- a/data/conf_snap_output/conf_snap_c.xlsx
+++ b/data/conf_snap_output/conf_snap_c.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -411,7 +411,7 @@
         <v>100</v>
       </c>
       <c r="B2">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="C2">
         <v>0.01</v>
@@ -426,16 +426,16 @@
         <v>0.05</v>
       </c>
       <c r="G2">
-        <v>0.06060606060606061</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="H2">
-        <v>0.9393939393939394</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I2">
-        <v>0.9340000000000001</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="J2">
-        <v>1000</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3">
@@ -443,7 +443,7 @@
         <v>100</v>
       </c>
       <c r="B3">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="C3">
         <v>0.05</v>
@@ -458,16 +458,16 @@
         <v>0.05</v>
       </c>
       <c r="G3">
-        <v>0.01265822784810127</v>
+        <v>0.5</v>
       </c>
       <c r="H3">
-        <v>0.9873417721518988</v>
+        <v>0.5</v>
       </c>
       <c r="I3">
-        <v>0.921</v>
+        <v>0.96</v>
       </c>
       <c r="J3">
-        <v>1000</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4">
@@ -475,7 +475,7 @@
         <v>100</v>
       </c>
       <c r="B4">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="C4">
         <v>0.1</v>
@@ -490,16 +490,16 @@
         <v>0.05</v>
       </c>
       <c r="G4">
-        <v>0.04</v>
+        <v>0.5</v>
       </c>
       <c r="H4">
+        <v>0.5</v>
+      </c>
+      <c r="I4">
         <v>0.96</v>
       </c>
-      <c r="I4">
-        <v>0.925</v>
-      </c>
       <c r="J4">
-        <v>1000</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
@@ -507,7 +507,7 @@
         <v>100</v>
       </c>
       <c r="B5">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="C5">
         <v>0.15</v>
@@ -522,16 +522,16 @@
         <v>0.05</v>
       </c>
       <c r="G5">
-        <v>0.01408450704225352</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="H5">
-        <v>0.9859154929577465</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I5">
-        <v>0.929</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="J5">
-        <v>1000</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6">
@@ -539,7 +539,7 @@
         <v>100</v>
       </c>
       <c r="B6">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="C6">
         <v>0.2</v>
@@ -554,16 +554,16 @@
         <v>0.05</v>
       </c>
       <c r="G6">
-        <v>0.01694915254237288</v>
+        <v>0</v>
       </c>
       <c r="H6">
-        <v>0.9830508474576272</v>
+        <v>1</v>
       </c>
       <c r="I6">
-        <v>0.9409999999999999</v>
+        <v>0.98</v>
       </c>
       <c r="J6">
-        <v>1000</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7">
@@ -571,7 +571,7 @@
         <v>100</v>
       </c>
       <c r="B7">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="C7">
         <v>0.25</v>
@@ -592,10 +592,10 @@
         <v>1</v>
       </c>
       <c r="I7">
-        <v>0.928</v>
+        <v>0.96</v>
       </c>
       <c r="J7">
-        <v>1000</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8">
@@ -603,10 +603,10 @@
         <v>100</v>
       </c>
       <c r="B8">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="C8">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="D8">
         <v>1000</v>
@@ -624,10 +624,10 @@
         <v>1</v>
       </c>
       <c r="I8">
-        <v>0.9340000000000001</v>
+        <v>0.96</v>
       </c>
       <c r="J8">
-        <v>1000</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9">
@@ -635,7 +635,7 @@
         <v>100</v>
       </c>
       <c r="B9">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="C9">
         <v>0.4</v>
@@ -650,144 +650,16 @@
         <v>0.05</v>
       </c>
       <c r="G9">
-        <v>0.01818181818181818</v>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>0.9818181818181818</v>
+        <v>1</v>
       </c>
       <c r="I9">
-        <v>0.945</v>
+        <v>0.96</v>
       </c>
       <c r="J9">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>100</v>
-      </c>
-      <c r="B10">
-        <v>0.02</v>
-      </c>
-      <c r="C10">
-        <v>0.5</v>
-      </c>
-      <c r="D10">
-        <v>1000</v>
-      </c>
-      <c r="E10">
-        <v>50</v>
-      </c>
-      <c r="F10">
-        <v>0.05</v>
-      </c>
-      <c r="G10">
-        <v>0</v>
-      </c>
-      <c r="H10">
-        <v>1</v>
-      </c>
-      <c r="I10">
-        <v>0.947</v>
-      </c>
-      <c r="J10">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>100</v>
-      </c>
-      <c r="B11">
-        <v>0.02</v>
-      </c>
-      <c r="C11">
-        <v>0.6</v>
-      </c>
-      <c r="D11">
-        <v>1000</v>
-      </c>
-      <c r="E11">
-        <v>50</v>
-      </c>
-      <c r="F11">
-        <v>0.05</v>
-      </c>
-      <c r="G11">
-        <v>0</v>
-      </c>
-      <c r="H11">
-        <v>1</v>
-      </c>
-      <c r="I11">
-        <v>0.9409999999999999</v>
-      </c>
-      <c r="J11">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <v>100</v>
-      </c>
-      <c r="B12">
-        <v>0.02</v>
-      </c>
-      <c r="C12">
-        <v>0.7</v>
-      </c>
-      <c r="D12">
-        <v>1000</v>
-      </c>
-      <c r="E12">
-        <v>50</v>
-      </c>
-      <c r="F12">
-        <v>0.05</v>
-      </c>
-      <c r="G12">
-        <v>0</v>
-      </c>
-      <c r="H12">
-        <v>1</v>
-      </c>
-      <c r="I12">
-        <v>0.953</v>
-      </c>
-      <c r="J12">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13">
-        <v>100</v>
-      </c>
-      <c r="B13">
-        <v>0.02</v>
-      </c>
-      <c r="C13">
-        <v>0.8</v>
-      </c>
-      <c r="D13">
-        <v>1000</v>
-      </c>
-      <c r="E13">
-        <v>50</v>
-      </c>
-      <c r="F13">
-        <v>0.05</v>
-      </c>
-      <c r="G13">
-        <v>0</v>
-      </c>
-      <c r="H13">
-        <v>1</v>
-      </c>
-      <c r="I13">
-        <v>0.949</v>
-      </c>
-      <c r="J13">
-        <v>1000</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>